<commit_message>
feat: company assumptions, waterfall dilution, Excel export, and new UI components
- Add Company Assumptions page with GET/PUT API endpoints for share counts,
  MIP, TSO/existing warrants, and PIK rate (synced across models)
- Replace parallel dilution with cascading waterfall model:
  MIP → TSO warrants → Existing warrants (each step updates PPS)
- Fix Excel export: correct ExcelJS definedNames API (location, name),
  fix calculateDealReturns 5-arg call, populate all 9 sheets
- Add Synergies Editor, Debt Schedule, Sensitivity Heatmap,
  Share Tracker, and Target Overview/Compare pages
- Enhance Capital Structure with source type classification and
  auto-derive ordinary/preferred equity and net debt from sources
- Expand Deal Returns Matrix with per-share and combined sections
- Add ErrorBoundary component for graceful error handling
</commit_message>
<xml_diff>
--- a/Div filer/Test Herjedal.xlsx
+++ b/Div filer/Test Herjedal.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrofasting/CODE/ECIT-acquisition/Div filer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EB3E969-293D-AA48-9C3D-2AE0E7CBC156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92C2EECE-54BE-8D4D-8071-A75762BCA378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="27660" windowHeight="18980" xr2:uid="{CD6F9456-AB92-5448-9CE2-F0C930A13991}"/>
+    <workbookView xWindow="0" yWindow="5200" windowWidth="23940" windowHeight="18980" xr2:uid="{CD6F9456-AB92-5448-9CE2-F0C930A13991}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>Argon (Sellside case)</t>
   </si>
@@ -70,16 +69,29 @@
   </si>
   <si>
     <t>EBITDA (pre IFRS)</t>
+  </si>
+  <si>
+    <t>Herjedal Buy side</t>
+  </si>
+  <si>
+    <t>Ebitda</t>
+  </si>
+  <si>
+    <t>Ebitda%</t>
+  </si>
+  <si>
+    <t>Organic growth</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0\ %"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0\ %"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -126,6 +138,13 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -144,10 +163,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -156,10 +176,17 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Prosent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -491,7 +518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA6FB135-D2ED-6547-B998-4E0EF4CCB5C2}">
-  <dimension ref="A3:I13"/>
+  <dimension ref="A3:I22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -701,31 +728,170 @@
         <v>4</v>
       </c>
       <c r="B13" s="8">
-        <f>B12/B9</f>
+        <f t="shared" ref="B13:G13" si="2">B12/B9</f>
         <v>0.12522045855379188</v>
       </c>
       <c r="C13" s="8">
-        <f>C12/C9</f>
+        <f t="shared" si="2"/>
         <v>0.12052117263843648</v>
       </c>
       <c r="D13" s="8">
-        <f>D12/D9</f>
+        <f t="shared" si="2"/>
         <v>0.11578947368421053</v>
       </c>
       <c r="E13" s="8">
-        <f>E12/E9</f>
+        <f t="shared" si="2"/>
         <v>0.12872628726287264</v>
       </c>
       <c r="F13" s="8">
-        <f>F12/F9</f>
+        <f t="shared" si="2"/>
         <v>0.14945321992709598</v>
       </c>
       <c r="G13" s="8">
-        <f>G12/G9</f>
+        <f t="shared" si="2"/>
         <v>0.17028199566160521</v>
       </c>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B18" s="7">
+        <f>B4</f>
+        <v>2025</v>
+      </c>
+      <c r="C18" s="7">
+        <f t="shared" ref="C18:G18" si="3">C4</f>
+        <v>2026</v>
+      </c>
+      <c r="D18" s="7">
+        <f t="shared" si="3"/>
+        <v>2027</v>
+      </c>
+      <c r="E18" s="7">
+        <f t="shared" si="3"/>
+        <v>2028</v>
+      </c>
+      <c r="F18" s="7">
+        <f t="shared" si="3"/>
+        <v>2029</v>
+      </c>
+      <c r="G18" s="7">
+        <f t="shared" si="3"/>
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="13">
+        <f>B9</f>
+        <v>567</v>
+      </c>
+      <c r="C19" s="13">
+        <f>B19*(1+C20)</f>
+        <v>538.65</v>
+      </c>
+      <c r="D19" s="13">
+        <f t="shared" ref="D19:G19" si="4">C19*(1+D20)</f>
+        <v>554.80949999999996</v>
+      </c>
+      <c r="E19" s="13">
+        <f t="shared" si="4"/>
+        <v>577.00188000000003</v>
+      </c>
+      <c r="F19" s="13">
+        <f t="shared" si="4"/>
+        <v>605.85197400000004</v>
+      </c>
+      <c r="G19" s="13">
+        <f t="shared" si="4"/>
+        <v>642.20309244000009</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" s="9">
+        <f>B21/B19</f>
+        <v>0.10229276895943562</v>
+      </c>
+      <c r="C20" s="11">
+        <v>-0.05</v>
+      </c>
+      <c r="D20" s="11">
+        <v>0.03</v>
+      </c>
+      <c r="E20" s="11">
+        <v>0.04</v>
+      </c>
+      <c r="F20" s="11">
+        <v>0.05</v>
+      </c>
+      <c r="G20" s="11">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" s="12">
+        <v>58</v>
+      </c>
+      <c r="C21" s="12">
+        <v>55</v>
+      </c>
+      <c r="D21" s="12">
+        <f>D19*D22</f>
+        <v>62.301094999999989</v>
+      </c>
+      <c r="E21" s="12">
+        <f t="shared" ref="E21:G21" si="5">E19*E22</f>
+        <v>70.563157599999997</v>
+      </c>
+      <c r="F21" s="12">
+        <f t="shared" si="5"/>
+        <v>80.14983522</v>
+      </c>
+      <c r="G21" s="12">
+        <f t="shared" si="5"/>
+        <v>83.486402017200021</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="10">
+        <f>B21/B19</f>
+        <v>0.10229276895943562</v>
+      </c>
+      <c r="C22" s="14">
+        <f>B22</f>
+        <v>0.10229276895943562</v>
+      </c>
+      <c r="D22" s="14">
+        <f>C22+1%</f>
+        <v>0.11229276895943562</v>
+      </c>
+      <c r="E22" s="14">
+        <f t="shared" ref="E22:F22" si="6">D22+1%</f>
+        <v>0.12229276895943561</v>
+      </c>
+      <c r="F22" s="14">
+        <f t="shared" si="6"/>
+        <v>0.13229276895943562</v>
+      </c>
+      <c r="G22" s="11">
+        <v>0.13</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>